<commit_message>
Feat: Add historical Excel logger for Export Sales, Inspections, WASDE and Crop Progress
</commit_message>
<xml_diff>
--- a/USDA Reports/CBOT_Reports_History.xlsx
+++ b/USDA Reports/CBOT_Reports_History.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J50"/>
+  <dimension ref="A1:J51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1141,6 +1141,34 @@
       <c r="I50" s="4" t="n"/>
       <c r="J50" s="4" t="n"/>
     </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>July 3-9, 2026</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>235.1</v>
+      </c>
+      <c r="C51" t="n">
+        <v>0</v>
+      </c>
+      <c r="D51" t="n">
+        <v>422.1</v>
+      </c>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="n">
+        <v>315</v>
+      </c>
+      <c r="H51" t="n">
+        <v>0</v>
+      </c>
+      <c r="I51" t="n">
+        <v>1588.3</v>
+      </c>
+      <c r="J51" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1152,7 +1180,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -1607,6 +1635,25 @@
       <c r="E50" s="4" t="n"/>
       <c r="F50" s="4" t="n"/>
     </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>JUL 16, 2026</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>213.993</v>
+      </c>
+      <c r="C51" t="n">
+        <v>-46</v>
+      </c>
+      <c r="E51" t="n">
+        <v>1549.849</v>
+      </c>
+      <c r="F51" t="n">
+        <v>-0.3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1618,7 +1665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K50"/>
+  <dimension ref="A1:K51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -2372,6 +2419,48 @@
       <c r="J50" s="4" t="n"/>
       <c r="K50" s="4" t="n"/>
     </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-07-20T12:00:00+0000</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>74% thu hoạch</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>N/A (Cuối vụ)</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>53% G/E</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>97% đã gieo trồng</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Mỹ: 0% | Argentina: 66% (2/3 tiến độ)</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>67% Good to Excellent</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2383,7 +2472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -2829,6 +2918,25 @@
       <c r="D50" s="6" t="n"/>
       <c r="E50" s="4" t="n"/>
       <c r="F50" s="4" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-07-10T12:00:00+0000</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>722</v>
+      </c>
+      <c r="C51" t="n">
+        <v>272.84</v>
+      </c>
+      <c r="E51" t="n">
+        <v>1790</v>
+      </c>
+      <c r="F51" t="n">
+        <v>275.26</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Auto sync: Dữ liệu Giá H1 + Macro mới
</commit_message>
<xml_diff>
--- a/USDA Reports/CBOT_Reports_History.xlsx
+++ b/USDA Reports/CBOT_Reports_History.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J29"/>
+  <dimension ref="A1:J30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -934,8 +934,6 @@
       <c r="D29" t="n">
         <v>422.1</v>
       </c>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
       <c r="G29" t="n">
         <v>315</v>
       </c>
@@ -945,7 +943,34 @@
       <c r="I29" t="n">
         <v>1588.3</v>
       </c>
-      <c r="J29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>July 10-16, 2026</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>290</v>
+      </c>
+      <c r="C30" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="D30" t="n">
+        <v>210.6</v>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="n">
+        <v>332.7</v>
+      </c>
+      <c r="H30" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="I30" t="n">
+        <v>1786.4</v>
+      </c>
+      <c r="J30" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Auto sync: Dữ liệu USDA Crop Progress mới
</commit_message>
<xml_diff>
--- a/USDA Reports/CBOT_Reports_History.xlsx
+++ b/USDA Reports/CBOT_Reports_History.xlsx
@@ -1009,8 +1009,6 @@
       <c r="D32" t="n">
         <v>319.2</v>
       </c>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
       <c r="G32" t="n">
         <v>362.9</v>
       </c>
@@ -1020,7 +1018,6 @@
       <c r="I32" t="n">
         <v>1528.5</v>
       </c>
-      <c r="J32" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1033,7 +1030,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -1364,6 +1361,26 @@
       </c>
       <c r="F29" t="n">
         <v>-7.7</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>JUL 30, 2026</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>335.313</v>
+      </c>
+      <c r="C30" t="n">
+        <v>-19.7</v>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="n">
+        <v>1884.68</v>
+      </c>
+      <c r="F30" t="n">
+        <v>22.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update: Export Sales 07/30/2026
</commit_message>
<xml_diff>
--- a/USDA Reports/CBOT_Reports_History.xlsx
+++ b/USDA Reports/CBOT_Reports_History.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:J33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1018,6 +1018,34 @@
       <c r="I32" t="n">
         <v>1528.5</v>
       </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>07/30/2026</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>296.4</v>
+      </c>
+      <c r="C33" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="D33" t="n">
+        <v>419</v>
+      </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="n">
+        <v>116.7</v>
+      </c>
+      <c r="H33" t="n">
+        <v>-67.8</v>
+      </c>
+      <c r="I33" t="n">
+        <v>1925.5</v>
+      </c>
+      <c r="J33" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2047,7 +2075,6 @@
           <t>2026-08-03T12:00:00+0000</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
           <t>86% thu hoạch</t>
@@ -2058,7 +2085,6 @@
           <t>N/A (Cuối vụ)</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
           <t>5% thu hoạch</t>
@@ -2069,7 +2095,6 @@
           <t>55% G/E</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
           <t>97% đã gieo trồng</t>

</xml_diff>

<commit_message>
Data: Export Sales 08/06/2026 - ZW 255.9k MT, ZC 410.7k MT
</commit_message>
<xml_diff>
--- a/USDA Reports/CBOT_Reports_History.xlsx
+++ b/USDA Reports/CBOT_Reports_History.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1043,6 +1043,34 @@
       <c r="I33" t="n">
         <v>1925.5</v>
       </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>08/06/2026</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>255.9</v>
+      </c>
+      <c r="C34" t="n">
+        <v>-13.7</v>
+      </c>
+      <c r="D34" t="n">
+        <v>490.6</v>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="n">
+        <v>410.7</v>
+      </c>
+      <c r="H34" t="n">
+        <v>251.9</v>
+      </c>
+      <c r="I34" t="n">
+        <v>1767.3</v>
+      </c>
+      <c r="J34" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2476,7 +2504,6 @@
       <c r="C28" t="n">
         <v>273.25</v>
       </c>
-      <c r="D28" t="inlineStr"/>
       <c r="E28" t="n">
         <v>1653</v>
       </c>

</xml_diff>

<commit_message>
Auto sync: Dữ liệu Export Sales mới
</commit_message>
<xml_diff>
--- a/USDA Reports/CBOT_Reports_History.xlsx
+++ b/USDA Reports/CBOT_Reports_History.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1068,6 +1068,34 @@
       <c r="I34" t="n">
         <v>1767.3</v>
       </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>08/13/2026</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>393.7</v>
+      </c>
+      <c r="C35" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="D35" t="n">
+        <v>524.3</v>
+      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="n">
+        <v>232.9</v>
+      </c>
+      <c r="H35" t="n">
+        <v>-43.3</v>
+      </c>
+      <c r="I35" t="n">
+        <v>1975.5</v>
+      </c>
+      <c r="J35" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1463,7 +1491,6 @@
       <c r="C32" t="n">
         <v>1.5</v>
       </c>
-      <c r="D32" t="inlineStr"/>
       <c r="E32" t="n">
         <v>1911</v>
       </c>

</xml_diff>